<commit_message>
Richer Telegram report: OI, Max Pain chart, levels with distances
- report sections: GEX (mode, conviction, pull status, walls / peak / pins
  with distance from price and dominant side, densest gamma just above and
  below the price, zero-gamma gaps inside the walls, a short reading) and
  Open Interest / Max Pain (zone, DTE, totals, P/C, top-3 call/put OI)
- second photo: call/put OI bars with the total-pain curve, price and Max Pain
- pain_by_strike() factored out of max_pain() for the chart
- "densest gamma" replaces the sheet's จุดหนืด column, whose 2x-median rule
  flags every strike when the median gross is 0 (as on 2026-10-07)
- fallback mode uses GEX Calc!J5's conviction rule instead of net > 0
- Telegram calls retry on timeout; Excel read-back retried once
- verify.excel_cells kills the COM-launched EXCEL.EXE it started (Quit()
  alone left 4 hidden instances running)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/คำนวน_max_pain_10 (2).xlsx
+++ b/คำนวน_max_pain_10 (2).xlsx
@@ -1007,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>AB1 Week 1 - OCT 2026 (V26)</t>
+          <t>WD1 Week 1 - OCT 2026 (V26)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -1027,13 +1027,13 @@
     </row>
     <row r="3" ht="25.5" customHeight="1" s="29">
       <c r="A3" s="2" t="n">
-        <v>3850</v>
+        <v>3800</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
@@ -1051,13 +1051,13 @@
     </row>
     <row r="4" ht="25.5" customHeight="1" s="29">
       <c r="A4" s="2" t="n">
-        <v>3875</v>
+        <v>3830</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="F4" s="26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -1075,13 +1075,13 @@
     </row>
     <row r="5" ht="25.5" customHeight="1" s="29">
       <c r="A5" s="2" t="n">
-        <v>3895</v>
+        <v>3900</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F5" s="26" t="n">
-        <v>1749</v>
+        <v>3129</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -1099,13 +1099,13 @@
     </row>
     <row r="6" ht="25.5" customHeight="1" s="29">
       <c r="A6" s="2" t="n">
-        <v>3900</v>
+        <v>3910</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="F6" s="26" t="n">
-        <v>1454</v>
+        <v>2068</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="7" ht="15" customHeight="1" s="29">
       <c r="A7" s="2" t="n">
-        <v>3915</v>
+        <v>3925</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
@@ -1140,287 +1140,287 @@
         <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="29">
       <c r="A9" s="2" t="n">
-        <v>3960</v>
+        <v>3955</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="29">
       <c r="A10" s="2" t="n">
-        <v>3975</v>
+        <v>3960</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="29">
       <c r="A11" s="2" t="n">
-        <v>3980</v>
+        <v>3970</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="2" t="n">
-        <v>3995</v>
+        <v>3975</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="2" t="n">
-        <v>4000</v>
+        <v>3980</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="2" t="n">
-        <v>4025</v>
+        <v>3995</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="29">
       <c r="A15" s="2" t="n">
-        <v>4035</v>
+        <v>4000</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="2" t="n">
-        <v>4045</v>
+        <v>4005</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="2" t="n">
-        <v>4050</v>
+        <v>4010</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="29">
       <c r="A18" s="2" t="n">
-        <v>4055</v>
+        <v>4020</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="29">
       <c r="A19" s="2" t="n">
-        <v>4060</v>
+        <v>4025</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="29">
       <c r="A20" s="2" t="n">
-        <v>4065</v>
+        <v>4035</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="29">
       <c r="A21" s="2" t="n">
-        <v>4070</v>
+        <v>4040</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="29">
       <c r="A22" s="2" t="n">
-        <v>4075</v>
+        <v>4045</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="29">
       <c r="A23" s="2" t="n">
-        <v>4080</v>
+        <v>4050</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="29">
       <c r="A24" s="2" t="n">
-        <v>4085</v>
+        <v>4055</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="29">
       <c r="A25" s="2" t="n">
-        <v>4090</v>
+        <v>4060</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="29">
       <c r="A26" s="2" t="n">
-        <v>4100</v>
+        <v>4065</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>259</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="29">
       <c r="A27" s="2" t="n">
-        <v>4105</v>
+        <v>4070</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="29">
       <c r="A28" s="2" t="n">
-        <v>4110</v>
+        <v>4075</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>9</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="29">
       <c r="A29" s="2" t="n">
-        <v>4115</v>
+        <v>4080</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="29">
       <c r="A30" s="2" t="n">
-        <v>4120</v>
+        <v>4085</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="29">
       <c r="A31" s="2" t="n">
-        <v>4125</v>
+        <v>4090</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="29">
       <c r="A32" s="2" t="n">
-        <v>4135</v>
+        <v>4095</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="29">
       <c r="A33" s="2" t="n">
-        <v>4140</v>
+        <v>4100</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>40</v>
+        <v>375</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="29">
       <c r="A34" s="2" t="n">
-        <v>4145</v>
+        <v>4105</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0</v>
@@ -1431,241 +1431,241 @@
     </row>
     <row r="35" ht="15" customHeight="1" s="29">
       <c r="A35" s="2" t="n">
-        <v>4150</v>
+        <v>4110</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="29">
       <c r="A36" s="2" t="n">
-        <v>4155</v>
+        <v>4115</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="29">
       <c r="A37" s="2" t="n">
-        <v>4160</v>
+        <v>4120</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>80</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="29">
       <c r="A38" s="2" t="n">
-        <v>4165</v>
+        <v>4125</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="29">
       <c r="A39" s="2" t="n">
-        <v>4170</v>
+        <v>4130</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>1</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="29">
       <c r="A40" s="2" t="n">
-        <v>4175</v>
+        <v>4135</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>209</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="29">
       <c r="A41" s="2" t="n">
-        <v>4180</v>
+        <v>4140</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="29">
       <c r="A42" s="2" t="n">
-        <v>4185</v>
+        <v>4145</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="29">
       <c r="A43" s="2" t="n">
-        <v>4190</v>
+        <v>4150</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>2</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="29">
       <c r="A44" s="2" t="n">
-        <v>4195</v>
+        <v>4155</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>111</v>
+        <v>3</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="29">
       <c r="A45" s="2" t="n">
-        <v>4200</v>
+        <v>4160</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>152</v>
+        <v>8</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="29">
       <c r="A46" s="2" t="n">
-        <v>4205</v>
+        <v>4165</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="29">
       <c r="A47" s="2" t="n">
-        <v>4210</v>
+        <v>4170</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="29">
       <c r="A48" s="2" t="n">
-        <v>4215</v>
+        <v>4175</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="29">
       <c r="A49" s="2" t="n">
-        <v>4220</v>
+        <v>4180</v>
       </c>
       <c r="B49" s="3" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="29">
       <c r="A50" s="2" t="n">
-        <v>4225</v>
+        <v>4185</v>
       </c>
       <c r="B50" s="3" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>63</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="29">
       <c r="A51" s="2" t="n">
-        <v>4230</v>
+        <v>4190</v>
       </c>
       <c r="B51" s="3" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="29">
       <c r="A52" s="2" t="n">
-        <v>4235</v>
+        <v>4195</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>4240</v>
+        <v>4200</v>
       </c>
       <c r="B53" s="3" t="n">
-        <v>12</v>
+        <v>109</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="29">
       <c r="A54" s="2" t="n">
-        <v>4245</v>
+        <v>4205</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="29">
       <c r="A55" s="2" t="n">
-        <v>4250</v>
+        <v>4210</v>
       </c>
       <c r="B55" s="3" t="n">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="29">
       <c r="A56" s="2" t="n">
-        <v>4255</v>
+        <v>4215</v>
       </c>
       <c r="B56" s="3" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C56" s="3" t="n">
         <v>0</v>
@@ -1673,32 +1673,32 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4260</v>
+        <v>4220</v>
       </c>
       <c r="B57" s="3" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4265</v>
+        <v>4225</v>
       </c>
       <c r="B58" s="3" t="n">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>4270</v>
+        <v>4230</v>
       </c>
       <c r="B59" s="3" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="C59" s="3" t="n">
         <v>0</v>
@@ -1706,21 +1706,21 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4275</v>
+        <v>4235</v>
       </c>
       <c r="B60" s="3" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4280</v>
+        <v>4240</v>
       </c>
       <c r="B61" s="3" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="C61" s="3" t="n">
         <v>0</v>
@@ -1728,32 +1728,32 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4285</v>
+        <v>4245</v>
       </c>
       <c r="B62" s="3" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4300</v>
+        <v>4250</v>
       </c>
       <c r="B63" t="n">
-        <v>67</v>
+        <v>321</v>
       </c>
       <c r="C63" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>4305</v>
+        <v>4255</v>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C64" t="n">
         <v>0</v>
@@ -1761,32 +1761,32 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>4310</v>
+        <v>4260</v>
       </c>
       <c r="B65" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>4315</v>
+        <v>4265</v>
       </c>
       <c r="B66" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4320</v>
+        <v>4270</v>
       </c>
       <c r="B67" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
@@ -1794,32 +1794,32 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4325</v>
+        <v>4275</v>
       </c>
       <c r="B68" t="n">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>162</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>4330</v>
+        <v>4280</v>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4340</v>
+        <v>4285</v>
       </c>
       <c r="B70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" t="n">
         <v>0</v>
@@ -1827,10 +1827,10 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4345</v>
+        <v>4290</v>
       </c>
       <c r="B71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" t="n">
         <v>0</v>
@@ -1838,10 +1838,10 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>4350</v>
+        <v>4295</v>
       </c>
       <c r="B72" t="n">
-        <v>119</v>
+        <v>3</v>
       </c>
       <c r="C72" t="n">
         <v>2</v>
@@ -1849,21 +1849,21 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4355</v>
+        <v>4300</v>
       </c>
       <c r="B73" t="n">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>4360</v>
+        <v>4305</v>
       </c>
       <c r="B74" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
@@ -1871,10 +1871,10 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>4365</v>
+        <v>4310</v>
       </c>
       <c r="B75" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C75" t="n">
         <v>0</v>
@@ -1882,10 +1882,10 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4370</v>
+        <v>4315</v>
       </c>
       <c r="B76" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C76" t="n">
         <v>0</v>
@@ -1893,54 +1893,54 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4375</v>
+        <v>4320</v>
       </c>
       <c r="B77" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>4380</v>
+        <v>4325</v>
       </c>
       <c r="B78" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>4385</v>
+        <v>4330</v>
       </c>
       <c r="B79" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>4400</v>
+        <v>4335</v>
       </c>
       <c r="B80" t="n">
-        <v>98</v>
+        <v>5</v>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>4410</v>
+        <v>4345</v>
       </c>
       <c r="B81" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
@@ -1948,21 +1948,21 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>4415</v>
+        <v>4350</v>
       </c>
       <c r="B82" t="n">
-        <v>5</v>
+        <v>401</v>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>4425</v>
+        <v>4365</v>
       </c>
       <c r="B83" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -1970,32 +1970,32 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>4450</v>
+        <v>4375</v>
       </c>
       <c r="B84" t="n">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>4475</v>
+        <v>4400</v>
       </c>
       <c r="B85" t="n">
-        <v>19</v>
+        <v>223</v>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>4500</v>
+        <v>4425</v>
       </c>
       <c r="B86" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
@@ -2003,21 +2003,21 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>4515</v>
+        <v>4450</v>
       </c>
       <c r="B87" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>4525</v>
+        <v>4475</v>
       </c>
       <c r="B88" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C88" t="n">
         <v>0</v>
@@ -2025,10 +2025,10 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>4550</v>
+        <v>4500</v>
       </c>
       <c r="B89" t="n">
-        <v>7</v>
+        <v>172</v>
       </c>
       <c r="C89" t="n">
         <v>0</v>
@@ -2036,21 +2036,21 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>4575</v>
+        <v>4525</v>
       </c>
       <c r="B90" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="C90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
       <c r="B91" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
@@ -2058,10 +2058,10 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>4625</v>
+        <v>4575</v>
       </c>
       <c r="B92" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C92" t="n">
         <v>0</v>
@@ -2069,10 +2069,10 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>4650</v>
+        <v>4600</v>
       </c>
       <c r="B93" t="n">
-        <v>19</v>
+        <v>254</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
@@ -2080,10 +2080,10 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>4675</v>
+        <v>4625</v>
       </c>
       <c r="B94" t="n">
-        <v>3</v>
+        <v>256</v>
       </c>
       <c r="C94" t="n">
         <v>0</v>
@@ -2091,10 +2091,10 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>4700</v>
+        <v>4650</v>
       </c>
       <c r="B95" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C95" t="n">
         <v>0</v>
@@ -2102,10 +2102,10 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>4725</v>
+        <v>4675</v>
       </c>
       <c r="B96" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C96" t="n">
         <v>0</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>4750</v>
+        <v>4700</v>
       </c>
       <c r="B97" t="n">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C97" t="n">
         <v>0</v>
@@ -2124,10 +2124,10 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>4775</v>
+        <v>4725</v>
       </c>
       <c r="B98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C98" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>4850</v>
+        <v>4750</v>
       </c>
       <c r="B99" t="n">
         <v>1</v>
@@ -2146,10 +2146,10 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>4900</v>
+        <v>4825</v>
       </c>
       <c r="B100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C100" t="n">
         <v>0</v>
@@ -2157,10 +2157,10 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>5100</v>
+        <v>4850</v>
       </c>
       <c r="B101" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C101" t="n">
         <v>0</v>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>5200</v>
+        <v>5100</v>
       </c>
       <c r="B102" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C102" t="n">
         <v>0</v>
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="F4" s="30" t="n">
-        <v>4162.3</v>
+        <v>4187.1</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="29">
@@ -5496,7 +5496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5934,9 +5934,53 @@
         </is>
       </c>
       <c r="K10" s="43" t="n">
-        <v>46301.38472030024</v>
+        <v>46301.38472030093</v>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>DEC 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WD1 Week 1 - OCT 2026 (V26)</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>4187.1</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>0.003080891309020476</v>
+      </c>
+      <c r="G11" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="39" t="n">
+        <v>0.6609140300415468</v>
+      </c>
+      <c r="I11" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>PRELIMINARY</t>
+        </is>
+      </c>
+      <c r="K11" s="43" t="n">
+        <v>46302.53311725874</v>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>DEC 26</t>
         </is>

</xml_diff>